<commit_message>
Update Excel export template with corrected background colors
</commit_message>
<xml_diff>
--- a/schedule-template.xlsx
+++ b/schedule-template.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91212F9B-0FD7-4BEA-AF9F-962947EB7382}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9838C3F-C958-4EDF-9333-9C91A1C6C436}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22944" yWindow="-84" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="班表資料" sheetId="5" r:id="rId1"/>
@@ -671,7 +671,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -715,12 +715,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFD9D9D9"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -914,14 +908,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -988,12 +979,6 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="176" fontId="8" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1015,16 +1000,19 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1353,46 +1341,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:35" ht="20.25" x14ac:dyDescent="0.25">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="31" t="s">
         <v>185</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37" t="s">
+      <c r="B1" s="31"/>
+      <c r="C1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="D1" s="31"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
     </row>
     <row r="2" spans="1:35" ht="18.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="22" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="23"/>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="23"/>
-      <c r="H2" s="23"/>
-      <c r="I2" s="23"/>
-      <c r="J2" s="23"/>
-      <c r="K2" s="23"/>
-      <c r="L2" s="23"/>
-      <c r="M2" s="23"/>
-      <c r="N2" s="23"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="23"/>
-      <c r="Q2" s="23"/>
-      <c r="R2" s="23"/>
-      <c r="S2" s="23"/>
-      <c r="T2" s="23"/>
-      <c r="U2" s="23"/>
-      <c r="V2" s="23"/>
-      <c r="W2" s="23"/>
-      <c r="X2" s="23"/>
-      <c r="Y2" s="23"/>
-      <c r="Z2" s="23"/>
+      <c r="B2" s="22"/>
+      <c r="C2" s="22"/>
+      <c r="D2" s="22"/>
+      <c r="E2" s="22"/>
+      <c r="F2" s="22"/>
+      <c r="G2" s="22"/>
+      <c r="H2" s="22"/>
+      <c r="I2" s="22"/>
+      <c r="J2" s="22"/>
+      <c r="K2" s="22"/>
+      <c r="L2" s="22"/>
+      <c r="M2" s="22"/>
+      <c r="N2" s="22"/>
+      <c r="O2" s="22"/>
+      <c r="P2" s="22"/>
+      <c r="Q2" s="22"/>
+      <c r="R2" s="22"/>
+      <c r="S2" s="22"/>
+      <c r="T2" s="22"/>
+      <c r="U2" s="22"/>
+      <c r="V2" s="22"/>
+      <c r="W2" s="22"/>
+      <c r="X2" s="22"/>
+      <c r="Y2" s="22"/>
+      <c r="Z2" s="22"/>
     </row>
     <row r="3" spans="1:35" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
@@ -1401,101 +1389,101 @@
       <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="24"/>
-      <c r="E3" s="34" t="s">
+      <c r="D3" s="23"/>
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="34" t="s">
+      <c r="F3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="34" t="s">
+      <c r="G3" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="H3" s="34" t="s">
+      <c r="H3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I3" s="34" t="s">
+      <c r="I3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J3" s="34" t="s">
+      <c r="J3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="K3" s="34" t="s">
+      <c r="K3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L3" s="34" t="s">
+      <c r="L3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="M3" s="34" t="s">
+      <c r="M3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="N3" s="34" t="s">
+      <c r="N3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="O3" s="34" t="s">
+      <c r="O3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="P3" s="34" t="s">
+      <c r="P3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="Q3" s="34" t="s">
+      <c r="Q3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="R3" s="34" t="s">
+      <c r="R3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="S3" s="34" t="s">
+      <c r="S3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="T3" s="34" t="s">
+      <c r="T3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="U3" s="34" t="s">
+      <c r="U3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="V3" s="34" t="s">
+      <c r="V3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="W3" s="34" t="s">
+      <c r="W3" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="X3" s="34" t="s">
+      <c r="X3" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="Y3" s="34" t="s">
+      <c r="Y3" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="Z3" s="34" t="s">
+      <c r="Z3" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="AA3" s="34" t="s">
+      <c r="AA3" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="AB3" s="34" t="s">
+      <c r="AB3" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="AC3" s="34" t="s">
+      <c r="AC3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AD3" s="34" t="s">
+      <c r="AD3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="AE3" s="34" t="s">
+      <c r="AE3" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="AF3" s="34" t="s">
+      <c r="AF3" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="AG3" s="34" t="s">
+      <c r="AG3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="AH3" s="34" t="s">
+      <c r="AH3" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="AI3" s="34" t="s">
+      <c r="AI3" s="1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1506,214 +1494,214 @@
       <c r="B4" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="34" t="s">
+      <c r="C4" s="23"/>
+      <c r="D4" s="23"/>
+      <c r="E4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="34" t="s">
+      <c r="F4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="G4" s="34" t="s">
+      <c r="G4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H4" s="34" t="s">
+      <c r="H4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I4" s="34" t="s">
+      <c r="I4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="J4" s="34" t="s">
+      <c r="J4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="K4" s="34" t="s">
+      <c r="K4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="34" t="s">
+      <c r="L4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="M4" s="34" t="s">
+      <c r="M4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="N4" s="34" t="s">
+      <c r="N4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="34" t="s">
+      <c r="O4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="P4" s="34" t="s">
+      <c r="P4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="34" t="s">
+      <c r="Q4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="R4" s="34" t="s">
+      <c r="R4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="S4" s="34" t="s">
+      <c r="S4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="T4" s="34" t="s">
+      <c r="T4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="U4" s="34" t="s">
+      <c r="U4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="V4" s="34" t="s">
+      <c r="V4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="W4" s="34" t="s">
+      <c r="W4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="X4" s="34" t="s">
+      <c r="X4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="Y4" s="34" t="s">
+      <c r="Y4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="Z4" s="34" t="s">
+      <c r="Z4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AA4" s="34" t="s">
+      <c r="AA4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AB4" s="34" t="s">
+      <c r="AB4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="AC4" s="34" t="s">
+      <c r="AC4" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AD4" s="34" t="s">
+      <c r="AD4" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="AE4" s="34" t="s">
+      <c r="AE4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="AF4" s="34" t="s">
+      <c r="AF4" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="AG4" s="34" t="s">
+      <c r="AG4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="AH4" s="34" t="s">
+      <c r="AH4" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="AI4" s="34" t="s">
+      <c r="AI4" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="36" t="s">
+      <c r="A5" s="32" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="32" t="s">
         <v>184</v>
       </c>
-      <c r="C5" s="25" t="s">
+      <c r="C5" s="33" t="s">
         <v>45</v>
       </c>
-      <c r="D5" s="25"/>
-      <c r="E5" s="35" t="s">
+      <c r="D5" s="33"/>
+      <c r="E5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="F5" s="35" t="s">
+      <c r="F5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="G5" s="35" t="s">
+      <c r="G5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="H5" s="35" t="s">
+      <c r="H5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="I5" s="35" t="s">
+      <c r="I5" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="J5" s="35" t="s">
+      <c r="J5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="K5" s="35" t="s">
+      <c r="K5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="L5" s="35" t="s">
+      <c r="L5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="M5" s="35" t="s">
+      <c r="M5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="N5" s="35" t="s">
+      <c r="N5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="O5" s="35" t="s">
+      <c r="O5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="P5" s="35" t="s">
+      <c r="P5" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="Q5" s="35" t="s">
+      <c r="Q5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="R5" s="35" t="s">
+      <c r="R5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="S5" s="35" t="s">
+      <c r="S5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="T5" s="35" t="s">
+      <c r="T5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="U5" s="35" t="s">
+      <c r="U5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="V5" s="35" t="s">
+      <c r="V5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="W5" s="35" t="s">
+      <c r="W5" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="X5" s="35" t="s">
+      <c r="X5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="Y5" s="35" t="s">
+      <c r="Y5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="Z5" s="35" t="s">
+      <c r="Z5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AA5" s="35" t="s">
+      <c r="AA5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AB5" s="35" t="s">
+      <c r="AB5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AC5" s="35" t="s">
+      <c r="AC5" s="34" t="s">
         <v>47</v>
       </c>
-      <c r="AD5" s="35" t="s">
+      <c r="AD5" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="AE5" s="35" t="s">
+      <c r="AE5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AF5" s="35" t="s">
+      <c r="AF5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AG5" s="35" t="s">
+      <c r="AG5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AH5" s="35" t="s">
+      <c r="AH5" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="AI5" s="35" t="s">
+      <c r="AI5" s="34" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="6" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="36"/>
-      <c r="B6" s="36"/>
-      <c r="C6" s="26" t="s">
+      <c r="A6" s="32"/>
+      <c r="B6" s="32"/>
+      <c r="C6" s="32" t="s">
         <v>49</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="35" t="s">
         <v>50</v>
       </c>
       <c r="E6" s="35" t="s">
@@ -1795,10 +1783,10 @@
       </c>
     </row>
     <row r="7" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="36"/>
-      <c r="B7" s="36"/>
-      <c r="C7" s="26"/>
-      <c r="D7" s="26" t="s">
+      <c r="A7" s="32"/>
+      <c r="B7" s="32"/>
+      <c r="C7" s="32"/>
+      <c r="D7" s="32" t="s">
         <v>52</v>
       </c>
       <c r="E7" s="35" t="s">
@@ -1838,10 +1826,10 @@
       <c r="AI7" s="35"/>
     </row>
     <row r="8" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="36"/>
-      <c r="B8" s="36"/>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
+      <c r="A8" s="32"/>
+      <c r="B8" s="32"/>
+      <c r="C8" s="32"/>
+      <c r="D8" s="32"/>
       <c r="E8" s="35" t="s">
         <v>138</v>
       </c>
@@ -1879,10 +1867,10 @@
       <c r="AI8" s="35"/>
     </row>
     <row r="9" spans="1:35" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="36"/>
-      <c r="B9" s="36"/>
-      <c r="C9" s="26"/>
-      <c r="D9" s="26"/>
+      <c r="A9" s="32"/>
+      <c r="B9" s="32"/>
+      <c r="C9" s="32"/>
+      <c r="D9" s="32"/>
       <c r="E9" s="35" t="s">
         <v>152</v>
       </c>
@@ -1965,243 +1953,243 @@
   <dimension ref="A1:L22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" style="3" customWidth="1"/>
-    <col min="2" max="2" width="15.42578125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="5.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" style="3" customWidth="1"/>
-    <col min="5" max="6" width="13.42578125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="15.140625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="9" style="3" customWidth="1"/>
-    <col min="9" max="16384" width="9" style="3"/>
+    <col min="1" max="1" width="9.42578125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="15.42578125" style="2" customWidth="1"/>
+    <col min="3" max="3" width="5.42578125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="9.85546875" style="2" customWidth="1"/>
+    <col min="5" max="6" width="13.42578125" style="2" customWidth="1"/>
+    <col min="7" max="7" width="15.140625" style="2" customWidth="1"/>
+    <col min="8" max="8" width="9" style="2" customWidth="1"/>
+    <col min="9" max="16384" width="9" style="2"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" ht="23.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="3" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
+      <c r="A2" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="6">
+      <c r="D2" s="25"/>
+      <c r="E2" s="5">
         <v>44409</v>
       </c>
-      <c r="F2" s="6">
+      <c r="F2" s="5">
         <v>44410</v>
       </c>
-      <c r="G2" s="6">
+      <c r="G2" s="5">
         <v>44411</v>
       </c>
     </row>
     <row r="3" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
+      <c r="A3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="B3" s="7" t="s">
+      <c r="B3" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="28"/>
-      <c r="E3" s="8" t="s">
+      <c r="C3" s="24"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F3" s="8" t="s">
+      <c r="F3" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G3" s="8" t="s">
+      <c r="G3" s="7" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="27" t="s">
         <v>56</v>
       </c>
-      <c r="B4" s="31" t="s">
+      <c r="B4" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="C4" s="29" t="s">
+      <c r="C4" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="D4" s="29"/>
-      <c r="E4" s="9" t="s">
+      <c r="D4" s="26"/>
+      <c r="E4" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="F4" s="10" t="s">
+      <c r="F4" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G4" s="10" t="s">
+      <c r="G4" s="9" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="30"/>
-      <c r="B5" s="32"/>
-      <c r="C5" s="31" t="s">
+      <c r="A5" s="27"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="28" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E5" s="12" t="s">
+      <c r="E5" s="11" t="s">
         <v>58</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="12" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="30"/>
-      <c r="B6" s="32"/>
-      <c r="C6" s="33"/>
-      <c r="D6" s="11" t="s">
+      <c r="A6" s="27"/>
+      <c r="B6" s="29"/>
+      <c r="C6" s="30"/>
+      <c r="D6" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E6" s="14" t="s">
+      <c r="E6" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="F6" s="15" t="s">
+      <c r="F6" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="G6" s="15" t="s">
+      <c r="G6" s="14" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="30"/>
-      <c r="B7" s="32"/>
-      <c r="C7" s="31" t="s">
+      <c r="A7" s="27"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="28" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="G7" s="12" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:12" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="30"/>
-      <c r="B8" s="33"/>
-      <c r="C8" s="33"/>
-      <c r="D8" s="11" t="s">
+      <c r="A8" s="27"/>
+      <c r="B8" s="30"/>
+      <c r="C8" s="30"/>
+      <c r="D8" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="15"/>
-      <c r="G8" s="15"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="14"/>
+      <c r="G8" s="14"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="16" t="s">
+      <c r="A10" s="15" t="s">
         <v>62</v>
       </c>
-      <c r="B10" s="17" t="s">
+      <c r="B10" s="16" t="s">
         <v>63</v>
       </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="17"/>
-      <c r="E10" s="17"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="17"/>
-      <c r="H10" s="17"/>
-      <c r="I10" s="17"/>
-      <c r="J10" s="17"/>
-      <c r="K10" s="17"/>
-      <c r="L10" s="17"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16"/>
+      <c r="K10" s="16"/>
+      <c r="L10" s="16"/>
     </row>
     <row r="11" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="18">
+      <c r="A11" s="17">
         <v>1</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="J11" s="19"/>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
     </row>
     <row r="12" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="20" t="s">
+      <c r="A12" s="19" t="s">
         <v>65</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="18"/>
     </row>
     <row r="13" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="20" t="s">
+      <c r="A13" s="19" t="s">
         <v>67</v>
       </c>
-      <c r="B13" s="19" t="s">
+      <c r="B13" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="C13" s="19"/>
-      <c r="D13" s="19"/>
-      <c r="E13" s="19"/>
-      <c r="F13" s="19"/>
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
     </row>
     <row r="14" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="20" t="s">
+      <c r="A14" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="B14" s="19" t="s">
+      <c r="B14" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="C14" s="19"/>
-      <c r="D14" s="19"/>
-      <c r="E14" s="19"/>
-      <c r="F14" s="19"/>
+      <c r="C14" s="18"/>
+      <c r="D14" s="18"/>
+      <c r="E14" s="18"/>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="18">
+      <c r="A15" s="17">
         <v>2</v>
       </c>
-      <c r="B15" s="19" t="s">
+      <c r="B15" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="C15" s="19"/>
-      <c r="D15" s="19"/>
-      <c r="E15" s="19"/>
-      <c r="F15" s="19"/>
+      <c r="C15" s="18"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="18"/>
+      <c r="F15" s="18"/>
     </row>
     <row r="16" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="18">
+      <c r="A16" s="17">
         <v>3</v>
       </c>
-      <c r="B16" s="19" t="s">
+      <c r="B16" s="18" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="18">
+      <c r="A17" s="17">
         <v>4</v>
       </c>
-      <c r="B17" s="19" t="s">
+      <c r="B17" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="19"/>
-      <c r="D17" s="19"/>
-      <c r="E17" s="19"/>
-      <c r="F17" s="19"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
     </row>
     <row r="22" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
@@ -2228,50 +2216,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="20" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>46</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>77</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>47</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2295,95 +2283,95 @@
     <col min="7" max="7" width="11.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D1" s="20" t="s">
         <v>82</v>
       </c>
-      <c r="E1" s="21" t="s">
+      <c r="E1" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="21" t="s">
+      <c r="F1" s="20" t="s">
         <v>84</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="20" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>85</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="D2" s="22" t="s">
+      <c r="D2" s="21" t="s">
         <v>87</v>
       </c>
-      <c r="E2" s="22" t="s">
+      <c r="E2" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="F2" s="22" t="s">
+      <c r="F2" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="G2" s="22" t="s">
+      <c r="G2" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="D3" s="22" t="s">
+      <c r="D3" s="21" t="s">
         <v>91</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="E3" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="F3" s="22" t="s">
+      <c r="F3" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="G3" s="22" t="s">
+      <c r="G3" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>92</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>93</v>
       </c>
-      <c r="D4" s="22" t="s">
+      <c r="D4" s="21" t="s">
         <v>94</v>
       </c>
-      <c r="E4" s="22" t="s">
+      <c r="E4" s="21" t="s">
         <v>88</v>
       </c>
-      <c r="F4" s="22" t="s">
+      <c r="F4" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="G4" s="21" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2405,530 +2393,530 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="21" t="s">
+      <c r="A1" s="20" t="s">
         <v>95</v>
       </c>
-      <c r="B1" s="21" t="s">
+      <c r="B1" s="20" t="s">
         <v>96</v>
       </c>
-      <c r="C1" s="21" t="s">
+      <c r="C1" s="20" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>97</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="21" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>99</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="21" t="s">
         <v>100</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="21" t="s">
         <v>103</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="C5" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="21" t="s">
         <v>104</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="21" t="s">
         <v>105</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="C6" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="21" t="s">
         <v>106</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="21" t="s">
         <v>107</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="C7" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="21" t="s">
         <v>108</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="21" t="s">
         <v>110</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="21" t="s">
         <v>111</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="C9" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="21" t="s">
         <v>112</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="C10" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="21" t="s">
         <v>114</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="B11" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="22" t="s">
+      <c r="A12" s="21" t="s">
         <v>116</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="B12" s="21" t="s">
         <v>117</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="C12" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="22" t="s">
+      <c r="A13" s="21" t="s">
         <v>118</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="B13" s="21" t="s">
         <v>119</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="C13" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="22" t="s">
+      <c r="A14" s="21" t="s">
         <v>120</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="21" t="s">
         <v>121</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="22" t="s">
+      <c r="A15" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>123</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="21" t="s">
         <v>124</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="21" t="s">
         <v>125</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" s="22" t="s">
+      <c r="A17" s="21" t="s">
         <v>126</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="B17" s="21" t="s">
         <v>127</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="C17" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" s="22" t="s">
+      <c r="A18" s="21" t="s">
         <v>128</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="B18" s="21" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="C18" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" s="22" t="s">
+      <c r="A19" s="21" t="s">
         <v>129</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="B19" s="21" t="s">
         <v>130</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="C19" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="22" t="s">
+      <c r="A20" s="21" t="s">
         <v>131</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="B20" s="21" t="s">
         <v>132</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="C20" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="22" t="s">
+      <c r="A21" s="21" t="s">
         <v>133</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="B21" s="21" t="s">
         <v>134</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="C21" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="22" t="s">
+      <c r="A22" s="21" t="s">
         <v>135</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="B22" s="21" t="s">
         <v>136</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="C22" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" s="22" t="s">
+      <c r="A23" s="21" t="s">
         <v>137</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="B23" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" s="22" t="s">
+      <c r="A24" s="21" t="s">
         <v>139</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="21" t="s">
         <v>140</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="C24" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" s="22" t="s">
+      <c r="A25" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="B25" s="21" t="s">
         <v>142</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="C25" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" s="22" t="s">
+      <c r="A26" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="B26" s="21" t="s">
         <v>143</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="C26" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="22" t="s">
+      <c r="A27" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="B27" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="C27" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="22" t="s">
+      <c r="A28" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="B28" s="22" t="s">
+      <c r="B28" s="21" t="s">
         <v>145</v>
       </c>
-      <c r="C28" s="22" t="s">
+      <c r="C28" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="22" t="s">
+      <c r="A29" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="B29" s="22" t="s">
+      <c r="B29" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="C29" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="22" t="s">
+      <c r="A30" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="B30" s="22" t="s">
+      <c r="B30" s="21" t="s">
         <v>147</v>
       </c>
-      <c r="C30" s="22" t="s">
+      <c r="C30" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="22" t="s">
+      <c r="A31" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="B31" s="22" t="s">
+      <c r="B31" s="21" t="s">
         <v>148</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="C31" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" s="22" t="s">
+      <c r="A32" s="21" t="s">
         <v>149</v>
       </c>
-      <c r="B32" s="22" t="s">
+      <c r="B32" s="21" t="s">
         <v>150</v>
       </c>
-      <c r="C32" s="22" t="s">
+      <c r="C32" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" s="22" t="s">
+      <c r="A33" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="B33" s="22" t="s">
+      <c r="B33" s="21" t="s">
         <v>152</v>
       </c>
-      <c r="C33" s="22" t="s">
+      <c r="C33" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" s="22" t="s">
+      <c r="A34" s="21" t="s">
         <v>153</v>
       </c>
-      <c r="B34" s="22" t="s">
+      <c r="B34" s="21" t="s">
         <v>154</v>
       </c>
-      <c r="C34" s="22" t="s">
+      <c r="C34" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" s="22" t="s">
+      <c r="A35" s="21" t="s">
         <v>155</v>
       </c>
-      <c r="B35" s="22" t="s">
+      <c r="B35" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="C35" s="22" t="s">
+      <c r="C35" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" s="22" t="s">
+      <c r="A36" s="21" t="s">
         <v>157</v>
       </c>
-      <c r="B36" s="22" t="s">
+      <c r="B36" s="21" t="s">
         <v>158</v>
       </c>
-      <c r="C36" s="22" t="s">
+      <c r="C36" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" s="22" t="s">
+      <c r="A37" s="21" t="s">
         <v>159</v>
       </c>
-      <c r="B37" s="22" t="s">
+      <c r="B37" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="C37" s="22" t="s">
+      <c r="C37" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" s="22" t="s">
+      <c r="A38" s="21" t="s">
         <v>161</v>
       </c>
-      <c r="B38" s="22" t="s">
+      <c r="B38" s="21" t="s">
         <v>162</v>
       </c>
-      <c r="C38" s="22" t="s">
+      <c r="C38" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="22" t="s">
+      <c r="A39" s="21" t="s">
         <v>163</v>
       </c>
-      <c r="B39" s="22" t="s">
+      <c r="B39" s="21" t="s">
         <v>164</v>
       </c>
-      <c r="C39" s="22" t="s">
+      <c r="C39" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" s="22" t="s">
+      <c r="A40" s="21" t="s">
         <v>165</v>
       </c>
-      <c r="B40" s="22" t="s">
+      <c r="B40" s="21" t="s">
         <v>166</v>
       </c>
-      <c r="C40" s="22" t="s">
+      <c r="C40" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" s="22" t="s">
+      <c r="A41" s="21" t="s">
         <v>167</v>
       </c>
-      <c r="B41" s="22" t="s">
+      <c r="B41" s="21" t="s">
         <v>168</v>
       </c>
-      <c r="C41" s="22" t="s">
+      <c r="C41" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" s="22" t="s">
+      <c r="A42" s="21" t="s">
         <v>169</v>
       </c>
-      <c r="B42" s="22" t="s">
+      <c r="B42" s="21" t="s">
         <v>170</v>
       </c>
-      <c r="C42" s="22" t="s">
+      <c r="C42" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" s="22" t="s">
+      <c r="A43" s="21" t="s">
         <v>171</v>
       </c>
-      <c r="B43" s="22" t="s">
+      <c r="B43" s="21" t="s">
         <v>172</v>
       </c>
-      <c r="C43" s="22" t="s">
+      <c r="C43" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" s="22" t="s">
+      <c r="A44" s="21" t="s">
         <v>173</v>
       </c>
-      <c r="B44" s="22" t="s">
+      <c r="B44" s="21" t="s">
         <v>174</v>
       </c>
-      <c r="C44" s="22" t="s">
+      <c r="C44" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" s="22" t="s">
+      <c r="A45" s="21" t="s">
         <v>175</v>
       </c>
-      <c r="B45" s="22" t="s">
+      <c r="B45" s="21" t="s">
         <v>176</v>
       </c>
-      <c r="C45" s="22" t="s">
+      <c r="C45" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" s="22" t="s">
+      <c r="A46" s="21" t="s">
         <v>177</v>
       </c>
-      <c r="B46" s="22" t="s">
+      <c r="B46" s="21" t="s">
         <v>178</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" s="22" t="s">
+      <c r="A47" s="21" t="s">
         <v>179</v>
       </c>
-      <c r="B47" s="22" t="s">
+      <c r="B47" s="21" t="s">
         <v>180</v>
       </c>
-      <c r="C47" s="22" t="s">
+      <c r="C47" s="21" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" s="22" t="s">
+      <c r="A48" s="21" t="s">
         <v>181</v>
       </c>
-      <c r="B48" s="22" t="s">
+      <c r="B48" s="21" t="s">
         <v>182</v>
       </c>
-      <c r="C48" s="22" t="s">
+      <c r="C48" s="21" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>